<commit_message>
fix: using num of buildings instead of dwellings
</commit_message>
<xml_diff>
--- a/exp/jack/Data/UK_Data/GB_Ambience.xlsx
+++ b/exp/jack/Data/UK_Data/GB_Ambience.xlsx
@@ -1,15 +1,34 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="11011"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/JackLynch/CUBES/exp/jack/Data/UK_Data/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15593438-9804-D94D-BF95-F0DA909AA778}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="240" yWindow="460" windowWidth="16100" windowHeight="9660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -316,8 +335,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -369,17 +388,26 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -426,7 +454,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
+        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -458,9 +486,27 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -492,6 +538,24 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -667,11 +731,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AZ28"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:BC28"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:52">
+    <row r="1" spans="1:55" x14ac:dyDescent="0.2">
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
@@ -826,7 +890,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="2" spans="1:52">
+    <row r="2" spans="1:55" x14ac:dyDescent="0.2">
       <c r="A2" s="1">
         <v>0</v>
       </c>
@@ -849,7 +913,7 @@
         <v>92</v>
       </c>
       <c r="H2">
-        <v>900000</v>
+        <v>220000.00000000003</v>
       </c>
       <c r="I2">
         <v>316.5</v>
@@ -915,7 +979,7 @@
         <v>0.2</v>
       </c>
       <c r="AD2">
-        <v>2.3</v>
+        <v>2.2999999999999998</v>
       </c>
       <c r="AE2">
         <v>0</v>
@@ -984,7 +1048,7 @@
         <v>316.5</v>
       </c>
     </row>
-    <row r="3" spans="1:52">
+    <row r="3" spans="1:55" x14ac:dyDescent="0.2">
       <c r="A3" s="1">
         <v>1</v>
       </c>
@@ -1007,7 +1071,7 @@
         <v>93</v>
       </c>
       <c r="H3">
-        <v>400000</v>
+        <v>92000</v>
       </c>
       <c r="I3">
         <v>360.13</v>
@@ -1016,7 +1080,7 @@
         <v>0</v>
       </c>
       <c r="K3">
-        <v>2250.57</v>
+        <v>2250.5700000000002</v>
       </c>
       <c r="L3">
         <v>0</v>
@@ -1109,7 +1173,7 @@
         <v>0</v>
       </c>
       <c r="AP3">
-        <v>0.012</v>
+        <v>1.2E-2</v>
       </c>
       <c r="AQ3">
         <v>0</v>
@@ -1133,7 +1197,7 @@
         <v>360.13</v>
       </c>
       <c r="AX3">
-        <v>2250.57</v>
+        <v>2250.5700000000002</v>
       </c>
       <c r="AY3">
         <v>912.41</v>
@@ -1142,7 +1206,7 @@
         <v>360.13</v>
       </c>
     </row>
-    <row r="4" spans="1:52">
+    <row r="4" spans="1:55" x14ac:dyDescent="0.2">
       <c r="A4" s="1">
         <v>2</v>
       </c>
@@ -1165,7 +1229,7 @@
         <v>93</v>
       </c>
       <c r="H4">
-        <v>700000</v>
+        <v>148000</v>
       </c>
       <c r="I4">
         <v>460.86</v>
@@ -1237,7 +1301,7 @@
         <v>0</v>
       </c>
       <c r="AF4">
-        <v>0.28</v>
+        <v>0.28000000000000003</v>
       </c>
       <c r="AG4">
         <v>0</v>
@@ -1300,7 +1364,7 @@
         <v>460.86</v>
       </c>
     </row>
-    <row r="5" spans="1:52">
+    <row r="5" spans="1:55" x14ac:dyDescent="0.2">
       <c r="A5" s="1">
         <v>3</v>
       </c>
@@ -1323,10 +1387,10 @@
         <v>92</v>
       </c>
       <c r="H5">
-        <v>1162225.114463213</v>
+        <v>508421.05263157887</v>
       </c>
       <c r="I5">
-        <v>149.11</v>
+        <v>149.11000000000001</v>
       </c>
       <c r="J5">
         <v>0</v>
@@ -1341,7 +1405,7 @@
         <v>0</v>
       </c>
       <c r="N5">
-        <v>69.79000000000001</v>
+        <v>69.790000000000006</v>
       </c>
       <c r="O5">
         <v>0</v>
@@ -1359,7 +1423,7 @@
         <v>0</v>
       </c>
       <c r="T5">
-        <v>149.11</v>
+        <v>149.11000000000001</v>
       </c>
       <c r="U5">
         <v>0</v>
@@ -1389,7 +1453,7 @@
         <v>0.2</v>
       </c>
       <c r="AD5">
-        <v>2.3</v>
+        <v>2.2999999999999998</v>
       </c>
       <c r="AE5">
         <v>0</v>
@@ -1446,19 +1510,20 @@
         <v>0</v>
       </c>
       <c r="AW5">
-        <v>149.11</v>
+        <v>149.11000000000001</v>
       </c>
       <c r="AX5">
         <v>233.3</v>
       </c>
       <c r="AY5">
-        <v>69.79000000000001</v>
+        <v>69.790000000000006</v>
       </c>
       <c r="AZ5">
-        <v>149.11</v>
-      </c>
+        <v>149.11000000000001</v>
+      </c>
+      <c r="BC5" s="2"/>
     </row>
-    <row r="6" spans="1:52">
+    <row r="6" spans="1:55" x14ac:dyDescent="0.2">
       <c r="A6" s="1">
         <v>4</v>
       </c>
@@ -1481,7 +1546,7 @@
         <v>92</v>
       </c>
       <c r="H6">
-        <v>437939.8982035295</v>
+        <v>191578.94736842104</v>
       </c>
       <c r="I6">
         <v>168.18</v>
@@ -1547,7 +1612,7 @@
         <v>0.2</v>
       </c>
       <c r="AD6">
-        <v>2.3</v>
+        <v>2.2999999999999998</v>
       </c>
       <c r="AE6">
         <v>0</v>
@@ -1615,8 +1680,9 @@
       <c r="AZ6">
         <v>168.18</v>
       </c>
+      <c r="BC6" s="2"/>
     </row>
-    <row r="7" spans="1:52">
+    <row r="7" spans="1:55" x14ac:dyDescent="0.2">
       <c r="A7" s="1">
         <v>5</v>
       </c>
@@ -1639,7 +1705,7 @@
         <v>92</v>
       </c>
       <c r="H7">
-        <v>435680.7715189124</v>
+        <v>200000</v>
       </c>
       <c r="I7">
         <v>156.66</v>
@@ -1705,7 +1771,7 @@
         <v>0.2</v>
       </c>
       <c r="AD7">
-        <v>2.3</v>
+        <v>2.2999999999999998</v>
       </c>
       <c r="AE7">
         <v>0</v>
@@ -1773,8 +1839,9 @@
       <c r="AZ7">
         <v>156.66</v>
       </c>
+      <c r="BC7" s="2"/>
     </row>
-    <row r="8" spans="1:52">
+    <row r="8" spans="1:55" x14ac:dyDescent="0.2">
       <c r="A8" s="1">
         <v>6</v>
       </c>
@@ -1797,7 +1864,7 @@
         <v>93</v>
       </c>
       <c r="H8">
-        <v>682539.2644494153</v>
+        <v>208000.00000000003</v>
       </c>
       <c r="I8">
         <v>195</v>
@@ -1899,7 +1966,7 @@
         <v>0</v>
       </c>
       <c r="AP8">
-        <v>0.012</v>
+        <v>1.2E-2</v>
       </c>
       <c r="AQ8">
         <v>0</v>
@@ -1931,8 +1998,9 @@
       <c r="AZ8">
         <v>195</v>
       </c>
+      <c r="BC8" s="2"/>
     </row>
-    <row r="9" spans="1:52">
+    <row r="9" spans="1:55" x14ac:dyDescent="0.2">
       <c r="A9" s="1">
         <v>7</v>
       </c>
@@ -1955,7 +2023,7 @@
         <v>93</v>
       </c>
       <c r="H9">
-        <v>347483.6525540717</v>
+        <v>79000.000000000015</v>
       </c>
       <c r="I9">
         <v>220.11</v>
@@ -2089,8 +2157,9 @@
       <c r="AZ9">
         <v>220.11</v>
       </c>
+      <c r="BC9" s="2"/>
     </row>
-    <row r="10" spans="1:52">
+    <row r="10" spans="1:55" x14ac:dyDescent="0.2">
       <c r="A10" s="1">
         <v>8</v>
       </c>
@@ -2113,7 +2182,7 @@
         <v>93</v>
       </c>
       <c r="H10">
-        <v>575461.8686426906</v>
+        <v>183000</v>
       </c>
       <c r="I10">
         <v>240.33</v>
@@ -2247,8 +2316,9 @@
       <c r="AZ10">
         <v>240.33</v>
       </c>
+      <c r="BC10" s="2"/>
     </row>
-    <row r="11" spans="1:52">
+    <row r="11" spans="1:55" x14ac:dyDescent="0.2">
       <c r="A11" s="1">
         <v>9</v>
       </c>
@@ -2271,7 +2341,7 @@
         <v>93</v>
       </c>
       <c r="H11">
-        <v>425482.1458570058</v>
+        <v>180000</v>
       </c>
       <c r="I11">
         <v>342.81</v>
@@ -2301,7 +2371,7 @@
         <v>0</v>
       </c>
       <c r="R11">
-        <v>76.48999999999999</v>
+        <v>76.489999999999995</v>
       </c>
       <c r="S11">
         <v>0</v>
@@ -2405,8 +2475,9 @@
       <c r="AZ11">
         <v>342.81</v>
       </c>
+      <c r="BC11" s="2"/>
     </row>
-    <row r="12" spans="1:52">
+    <row r="12" spans="1:55" x14ac:dyDescent="0.2">
       <c r="A12" s="1">
         <v>10</v>
       </c>
@@ -2429,7 +2500,7 @@
         <v>93</v>
       </c>
       <c r="H12">
-        <v>406665.8146736709</v>
+        <v>200000.00000000006</v>
       </c>
       <c r="I12">
         <v>342.82</v>
@@ -2501,7 +2572,7 @@
         <v>0</v>
       </c>
       <c r="AF12">
-        <v>0.28</v>
+        <v>0.28000000000000003</v>
       </c>
       <c r="AG12">
         <v>0</v>
@@ -2563,8 +2634,9 @@
       <c r="AZ12">
         <v>342.82</v>
       </c>
+      <c r="BC12" s="2"/>
     </row>
-    <row r="13" spans="1:52">
+    <row r="13" spans="1:55" x14ac:dyDescent="0.2">
       <c r="A13" s="1">
         <v>11</v>
       </c>
@@ -2587,7 +2659,7 @@
         <v>92</v>
       </c>
       <c r="H13">
-        <v>2584603.245421711</v>
+        <v>1557947.368421053</v>
       </c>
       <c r="I13">
         <v>113.45</v>
@@ -2653,7 +2725,7 @@
         <v>0.2</v>
       </c>
       <c r="AD13">
-        <v>2.3</v>
+        <v>2.2999999999999998</v>
       </c>
       <c r="AE13">
         <v>0</v>
@@ -2721,8 +2793,9 @@
       <c r="AZ13">
         <v>113.45</v>
       </c>
+      <c r="BC13" s="2"/>
     </row>
-    <row r="14" spans="1:52">
+    <row r="14" spans="1:55" x14ac:dyDescent="0.2">
       <c r="A14" s="1">
         <v>12</v>
       </c>
@@ -2745,10 +2818,10 @@
         <v>92</v>
       </c>
       <c r="H14">
-        <v>973908.4692893407</v>
+        <v>587052.63157894753</v>
       </c>
       <c r="I14">
-        <v>97.56999999999999</v>
+        <v>97.57</v>
       </c>
       <c r="J14">
         <v>0</v>
@@ -2781,7 +2854,7 @@
         <v>0</v>
       </c>
       <c r="T14">
-        <v>97.56999999999999</v>
+        <v>97.57</v>
       </c>
       <c r="U14">
         <v>0</v>
@@ -2811,7 +2884,7 @@
         <v>0.2</v>
       </c>
       <c r="AD14">
-        <v>2.3</v>
+        <v>2.2999999999999998</v>
       </c>
       <c r="AE14">
         <v>0</v>
@@ -2868,7 +2941,7 @@
         <v>0</v>
       </c>
       <c r="AW14">
-        <v>97.56999999999999</v>
+        <v>97.57</v>
       </c>
       <c r="AX14">
         <v>155.32</v>
@@ -2877,10 +2950,11 @@
         <v>40.36</v>
       </c>
       <c r="AZ14">
-        <v>97.56999999999999</v>
-      </c>
+        <v>97.57</v>
+      </c>
+      <c r="BC14" s="2"/>
     </row>
-    <row r="15" spans="1:52">
+    <row r="15" spans="1:55" x14ac:dyDescent="0.2">
       <c r="A15" s="1">
         <v>13</v>
       </c>
@@ -2903,10 +2977,10 @@
         <v>92</v>
       </c>
       <c r="H15">
-        <v>2016979.437660281</v>
+        <v>1248000</v>
       </c>
       <c r="I15">
-        <v>97.31999999999999</v>
+        <v>97.32</v>
       </c>
       <c r="J15">
         <v>0</v>
@@ -2921,7 +2995,7 @@
         <v>0</v>
       </c>
       <c r="N15">
-        <v>35.3</v>
+        <v>35.299999999999997</v>
       </c>
       <c r="O15">
         <v>0</v>
@@ -2933,13 +3007,13 @@
         <v>0</v>
       </c>
       <c r="R15">
-        <v>18.1</v>
+        <v>18.100000000000001</v>
       </c>
       <c r="S15">
         <v>0</v>
       </c>
       <c r="T15">
-        <v>97.31999999999999</v>
+        <v>97.32</v>
       </c>
       <c r="U15">
         <v>0</v>
@@ -2969,7 +3043,7 @@
         <v>0.2</v>
       </c>
       <c r="AD15">
-        <v>2.3</v>
+        <v>2.2999999999999998</v>
       </c>
       <c r="AE15">
         <v>0</v>
@@ -3026,19 +3100,20 @@
         <v>0</v>
       </c>
       <c r="AW15">
-        <v>97.31999999999999</v>
+        <v>97.32</v>
       </c>
       <c r="AX15">
         <v>134.1</v>
       </c>
       <c r="AY15">
-        <v>35.3</v>
+        <v>35.299999999999997</v>
       </c>
       <c r="AZ15">
-        <v>97.31999999999999</v>
-      </c>
+        <v>97.32</v>
+      </c>
+      <c r="BC15" s="2"/>
     </row>
-    <row r="16" spans="1:52">
+    <row r="16" spans="1:55" x14ac:dyDescent="0.2">
       <c r="A16" s="1">
         <v>14</v>
       </c>
@@ -3061,7 +3136,7 @@
         <v>93</v>
       </c>
       <c r="H16">
-        <v>1528402.40630546</v>
+        <v>1044999.9999999999</v>
       </c>
       <c r="I16">
         <v>86.89</v>
@@ -3163,7 +3238,7 @@
         <v>0</v>
       </c>
       <c r="AP16">
-        <v>0.012</v>
+        <v>1.2E-2</v>
       </c>
       <c r="AQ16">
         <v>0</v>
@@ -3195,8 +3270,9 @@
       <c r="AZ16">
         <v>86.89</v>
       </c>
+      <c r="BC16" s="2"/>
     </row>
-    <row r="17" spans="1:52">
+    <row r="17" spans="1:55" x14ac:dyDescent="0.2">
       <c r="A17" s="1">
         <v>15</v>
       </c>
@@ -3219,7 +3295,7 @@
         <v>93</v>
       </c>
       <c r="H17">
-        <v>690635.3254416462</v>
+        <v>529500</v>
       </c>
       <c r="I17">
         <v>82.36</v>
@@ -3228,7 +3304,7 @@
         <v>0</v>
       </c>
       <c r="K17">
-        <v>152.2</v>
+        <v>152.19999999999999</v>
       </c>
       <c r="L17">
         <v>0</v>
@@ -3345,7 +3421,7 @@
         <v>82.36</v>
       </c>
       <c r="AX17">
-        <v>152.2</v>
+        <v>152.19999999999999</v>
       </c>
       <c r="AY17">
         <v>30.4</v>
@@ -3353,8 +3429,9 @@
       <c r="AZ17">
         <v>82.36</v>
       </c>
+      <c r="BC17" s="2"/>
     </row>
-    <row r="18" spans="1:52">
+    <row r="18" spans="1:55" x14ac:dyDescent="0.2">
       <c r="A18" s="1">
         <v>16</v>
       </c>
@@ -3377,7 +3454,7 @@
         <v>93</v>
       </c>
       <c r="H18">
-        <v>1413108.196579827</v>
+        <v>976499.99999999988</v>
       </c>
       <c r="I18">
         <v>84.56</v>
@@ -3395,7 +3472,7 @@
         <v>0</v>
       </c>
       <c r="N18">
-        <v>34.2</v>
+        <v>34.200000000000003</v>
       </c>
       <c r="O18">
         <v>0</v>
@@ -3506,13 +3583,14 @@
         <v>166.8</v>
       </c>
       <c r="AY18">
-        <v>34.2</v>
+        <v>34.200000000000003</v>
       </c>
       <c r="AZ18">
         <v>84.56</v>
       </c>
+      <c r="BC18" s="2"/>
     </row>
-    <row r="19" spans="1:52">
+    <row r="19" spans="1:55" x14ac:dyDescent="0.2">
       <c r="A19" s="1">
         <v>17</v>
       </c>
@@ -3535,7 +3613,7 @@
         <v>93</v>
       </c>
       <c r="H19">
-        <v>1196256.657282985</v>
+        <v>756000</v>
       </c>
       <c r="I19">
         <v>86.92</v>
@@ -3565,7 +3643,7 @@
         <v>0</v>
       </c>
       <c r="R19">
-        <v>17.4</v>
+        <v>17.399999999999999</v>
       </c>
       <c r="S19">
         <v>0</v>
@@ -3669,8 +3747,9 @@
       <c r="AZ19">
         <v>86.92</v>
       </c>
+      <c r="BC19" s="2"/>
     </row>
-    <row r="20" spans="1:52">
+    <row r="20" spans="1:55" x14ac:dyDescent="0.2">
       <c r="A20" s="1">
         <v>18</v>
       </c>
@@ -3693,7 +3772,7 @@
         <v>93</v>
       </c>
       <c r="H20">
-        <v>1544366.996837492</v>
+        <v>1010000</v>
       </c>
       <c r="I20">
         <v>86.92</v>
@@ -3717,13 +3796,13 @@
         <v>0</v>
       </c>
       <c r="P20">
-        <v>18.1</v>
+        <v>18.100000000000001</v>
       </c>
       <c r="Q20">
         <v>0</v>
       </c>
       <c r="R20">
-        <v>17.4</v>
+        <v>17.399999999999999</v>
       </c>
       <c r="S20">
         <v>0</v>
@@ -3765,7 +3844,7 @@
         <v>0</v>
       </c>
       <c r="AF20">
-        <v>0.28</v>
+        <v>0.28000000000000003</v>
       </c>
       <c r="AG20">
         <v>0</v>
@@ -3827,8 +3906,9 @@
       <c r="AZ20">
         <v>86.92</v>
       </c>
+      <c r="BC20" s="2"/>
     </row>
-    <row r="21" spans="1:52">
+    <row r="21" spans="1:55" x14ac:dyDescent="0.2">
       <c r="A21" s="1">
         <v>19</v>
       </c>
@@ -3851,7 +3931,7 @@
         <v>92</v>
       </c>
       <c r="H21">
-        <v>2584603.245421711</v>
+        <v>1557947.368421053</v>
       </c>
       <c r="I21">
         <v>56.35</v>
@@ -3860,7 +3940,7 @@
         <v>0</v>
       </c>
       <c r="K21">
-        <v>89.09999999999999</v>
+        <v>89.1</v>
       </c>
       <c r="L21">
         <v>0</v>
@@ -3917,7 +3997,7 @@
         <v>0.2</v>
       </c>
       <c r="AD21">
-        <v>2.3</v>
+        <v>2.2999999999999998</v>
       </c>
       <c r="AE21">
         <v>0</v>
@@ -3977,7 +4057,7 @@
         <v>56.35</v>
       </c>
       <c r="AX21">
-        <v>89.09999999999999</v>
+        <v>89.1</v>
       </c>
       <c r="AY21">
         <v>24</v>
@@ -3985,8 +4065,9 @@
       <c r="AZ21">
         <v>56.35</v>
       </c>
+      <c r="BC21" s="2"/>
     </row>
-    <row r="22" spans="1:52">
+    <row r="22" spans="1:55" x14ac:dyDescent="0.2">
       <c r="A22" s="1">
         <v>20</v>
       </c>
@@ -4009,7 +4090,7 @@
         <v>92</v>
       </c>
       <c r="H22">
-        <v>973908.4692893407</v>
+        <v>587052.63157894753</v>
       </c>
       <c r="I22">
         <v>53.46</v>
@@ -4018,7 +4099,7 @@
         <v>0</v>
       </c>
       <c r="K22">
-        <v>87.59999999999999</v>
+        <v>87.6</v>
       </c>
       <c r="L22">
         <v>0</v>
@@ -4075,7 +4156,7 @@
         <v>0.2</v>
       </c>
       <c r="AD22">
-        <v>2.3</v>
+        <v>2.2999999999999998</v>
       </c>
       <c r="AE22">
         <v>0</v>
@@ -4135,7 +4216,7 @@
         <v>53.46</v>
       </c>
       <c r="AX22">
-        <v>87.59999999999999</v>
+        <v>87.6</v>
       </c>
       <c r="AY22">
         <v>25.4</v>
@@ -4143,8 +4224,9 @@
       <c r="AZ22">
         <v>53.46</v>
       </c>
+      <c r="BC22" s="2"/>
     </row>
-    <row r="23" spans="1:52">
+    <row r="23" spans="1:55" x14ac:dyDescent="0.2">
       <c r="A23" s="1">
         <v>21</v>
       </c>
@@ -4167,7 +4249,7 @@
         <v>92</v>
       </c>
       <c r="H23">
-        <v>2016979.437660281</v>
+        <v>1248000</v>
       </c>
       <c r="I23">
         <v>52.96</v>
@@ -4233,7 +4315,7 @@
         <v>0.2</v>
       </c>
       <c r="AD23">
-        <v>2.3</v>
+        <v>2.2999999999999998</v>
       </c>
       <c r="AE23">
         <v>0</v>
@@ -4301,8 +4383,9 @@
       <c r="AZ23">
         <v>52.96</v>
       </c>
+      <c r="BC23" s="2"/>
     </row>
-    <row r="24" spans="1:52">
+    <row r="24" spans="1:55" x14ac:dyDescent="0.2">
       <c r="A24" s="1">
         <v>22</v>
       </c>
@@ -4325,7 +4408,7 @@
         <v>93</v>
       </c>
       <c r="H24">
-        <v>1528402.40630546</v>
+        <v>1044999.9999999999</v>
       </c>
       <c r="I24">
         <v>51.94</v>
@@ -4427,7 +4510,7 @@
         <v>0</v>
       </c>
       <c r="AP24">
-        <v>0.012</v>
+        <v>1.2E-2</v>
       </c>
       <c r="AQ24">
         <v>0</v>
@@ -4459,8 +4542,9 @@
       <c r="AZ24">
         <v>51.94</v>
       </c>
+      <c r="BC24" s="2"/>
     </row>
-    <row r="25" spans="1:52">
+    <row r="25" spans="1:55" x14ac:dyDescent="0.2">
       <c r="A25" s="1">
         <v>23</v>
       </c>
@@ -4483,7 +4567,7 @@
         <v>93</v>
       </c>
       <c r="H25">
-        <v>690635.3254416462</v>
+        <v>529500</v>
       </c>
       <c r="I25">
         <v>44.3</v>
@@ -4492,7 +4576,7 @@
         <v>0</v>
       </c>
       <c r="K25">
-        <v>73.81999999999999</v>
+        <v>73.819999999999993</v>
       </c>
       <c r="L25">
         <v>0</v>
@@ -4501,19 +4585,19 @@
         <v>0</v>
       </c>
       <c r="N25">
-        <v>16.76</v>
+        <v>16.760000000000002</v>
       </c>
       <c r="O25">
         <v>0</v>
       </c>
       <c r="P25">
-        <v>8.720000000000001</v>
+        <v>8.7200000000000006</v>
       </c>
       <c r="Q25">
         <v>0</v>
       </c>
       <c r="R25">
-        <v>8.039999999999999</v>
+        <v>8.0399999999999991</v>
       </c>
       <c r="S25">
         <v>0</v>
@@ -4609,16 +4693,17 @@
         <v>44.3</v>
       </c>
       <c r="AX25">
-        <v>73.81999999999999</v>
+        <v>73.819999999999993</v>
       </c>
       <c r="AY25">
-        <v>16.76</v>
+        <v>16.760000000000002</v>
       </c>
       <c r="AZ25">
         <v>44.3</v>
       </c>
+      <c r="BC25" s="2"/>
     </row>
-    <row r="26" spans="1:52">
+    <row r="26" spans="1:55" x14ac:dyDescent="0.2">
       <c r="A26" s="1">
         <v>24</v>
       </c>
@@ -4641,7 +4726,7 @@
         <v>93</v>
       </c>
       <c r="H26">
-        <v>1413108.196579827</v>
+        <v>976499.99999999988</v>
       </c>
       <c r="I26">
         <v>44.31</v>
@@ -4650,7 +4735,7 @@
         <v>0</v>
       </c>
       <c r="K26">
-        <v>81.20999999999999</v>
+        <v>81.209999999999994</v>
       </c>
       <c r="L26">
         <v>0</v>
@@ -4767,7 +4852,7 @@
         <v>44.31</v>
       </c>
       <c r="AX26">
-        <v>81.20999999999999</v>
+        <v>81.209999999999994</v>
       </c>
       <c r="AY26">
         <v>17.59</v>
@@ -4775,8 +4860,9 @@
       <c r="AZ26">
         <v>44.31</v>
       </c>
+      <c r="BC26" s="2"/>
     </row>
-    <row r="27" spans="1:52">
+    <row r="27" spans="1:55" x14ac:dyDescent="0.2">
       <c r="A27" s="1">
         <v>25</v>
       </c>
@@ -4799,7 +4885,7 @@
         <v>93</v>
       </c>
       <c r="H27">
-        <v>1196256.657282985</v>
+        <v>756000</v>
       </c>
       <c r="I27">
         <v>47.27</v>
@@ -4808,7 +4894,7 @@
         <v>0</v>
       </c>
       <c r="K27">
-        <v>87.48999999999999</v>
+        <v>87.49</v>
       </c>
       <c r="L27">
         <v>0</v>
@@ -4925,7 +5011,7 @@
         <v>47.27</v>
       </c>
       <c r="AX27">
-        <v>87.48999999999999</v>
+        <v>87.49</v>
       </c>
       <c r="AY27">
         <v>19.39</v>
@@ -4933,8 +5019,9 @@
       <c r="AZ27">
         <v>47.27</v>
       </c>
+      <c r="BC27" s="2"/>
     </row>
-    <row r="28" spans="1:52">
+    <row r="28" spans="1:55" x14ac:dyDescent="0.2">
       <c r="A28" s="1">
         <v>26</v>
       </c>
@@ -4957,7 +5044,7 @@
         <v>93</v>
       </c>
       <c r="H28">
-        <v>1544366.996837492</v>
+        <v>1010000</v>
       </c>
       <c r="I28">
         <v>47.27</v>
@@ -4975,7 +5062,7 @@
         <v>0</v>
       </c>
       <c r="N28">
-        <v>19.4</v>
+        <v>19.399999999999999</v>
       </c>
       <c r="O28">
         <v>0</v>
@@ -5029,7 +5116,7 @@
         <v>0</v>
       </c>
       <c r="AF28">
-        <v>0.28</v>
+        <v>0.28000000000000003</v>
       </c>
       <c r="AG28">
         <v>0</v>
@@ -5086,11 +5173,12 @@
         <v>87.5</v>
       </c>
       <c r="AY28">
-        <v>19.4</v>
+        <v>19.399999999999999</v>
       </c>
       <c r="AZ28">
         <v>47.27</v>
       </c>
+      <c r="BC28" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>